<commit_message>
remove https://www.autoankauf-mainburg.de from excel
</commit_message>
<xml_diff>
--- a/src/test/resources/excelData.xlsx
+++ b/src/test/resources/excelData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\IdeaProjects\webseit-test\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7547ABB4-083F-4296-ADB6-EB443792BBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06DF4C83-CE19-4286-9328-FA032687CF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1A0E7E13-4B51-4D68-A319-BB2E1A6F5F75}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="362">
   <si>
     <t>auto-ankauf-warendorf.de</t>
   </si>
@@ -256,9 +256,6 @@
   </si>
   <si>
     <t>autoankauf-ratzeburg.de</t>
-  </si>
-  <si>
-    <t>autoankauf-mainburg.de</t>
   </si>
   <si>
     <t>autoankauf-bad-wildungen.de</t>
@@ -1566,7 +1563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87EF5093-2B8D-4748-B826-5F7196BA71A3}">
-  <dimension ref="A1:B363"/>
+  <dimension ref="A1:B362"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="51.44140625" customWidth="1"/>
@@ -1579,7 +1576,7 @@
         <v>https://www.amjis.com</v>
       </c>
       <c r="B1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1588,7 +1585,7 @@
         <v>https://www.key.stonepulse.com</v>
       </c>
       <c r="B2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1597,7 +1594,7 @@
         <v>https://www.kalender.stonepulse.com</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1606,7 +1603,7 @@
         <v>https://www.todo.stonepulse.com</v>
       </c>
       <c r="B4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1615,7 +1612,7 @@
         <v>https://www.ilamecca.com</v>
       </c>
       <c r="B5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -1624,7 +1621,7 @@
         <v>https://www.nivontec.de</v>
       </c>
       <c r="B6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1633,7 +1630,7 @@
         <v>https://www.nma-hamburg.de</v>
       </c>
       <c r="B7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -1642,7 +1639,7 @@
         <v>https://www.smarttech-elektro.de</v>
       </c>
       <c r="B8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -1651,7 +1648,7 @@
         <v>https://dr-elrafei.de</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1732,7 +1729,7 @@
         <v>https://www.autoankauf-wismar.de</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1768,7 +1765,7 @@
         <v>https://www.autoankauf-hanau.de</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1777,7 +1774,7 @@
         <v>https://www.autoankauf-celle.de</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1786,7 +1783,7 @@
         <v>https://www.autoankauf-saarlouis.de</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1795,7 +1792,7 @@
         <v>https://www.auto-ankauf-kiel.de</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1822,7 +1819,7 @@
         <v>https://www.dortmund-auto-ankauf.de</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1921,7 +1918,7 @@
         <v>https://www.kfz-ankauf-neubrandenburg.de</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1930,7 +1927,7 @@
         <v>https://www.autoankauf-schwerin.de</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1939,7 +1936,7 @@
         <v>https://www.autoankauf-emsland.de</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1948,7 +1945,7 @@
         <v>https://www.hannover-autoankauf.de</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1957,7 +1954,7 @@
         <v>https://www.oldenburg-auto-ankauf.de</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1966,7 +1963,7 @@
         <v>https://www.autoankauf-uelzen.de</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1975,7 +1972,7 @@
         <v>https://www.autoankauf-bad-oldesloe.de</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1984,7 +1981,7 @@
         <v>https://www.autoankauf-itzehoe.de</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -1993,7 +1990,7 @@
         <v>https://www.kfz-ankauf-kiel.de</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2002,7 +1999,7 @@
         <v>https://www.auto-ankauf-pinneberg.de</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2011,7 +2008,7 @@
         <v>https://www.auto-ankauf-straubing.de</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2020,7 +2017,7 @@
         <v>https://www.autoankauf-bad-nauheim.de</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2047,7 +2044,7 @@
         <v>https://www.autoankauf-gifhorn.de</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2056,7 +2053,7 @@
         <v>https://www.goslar-auto-ankauf.de</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2065,7 +2062,7 @@
         <v>https://www.autoankauf-helmstedt.de</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2074,7 +2071,7 @@
         <v>https://www.auto-ankauf-meppen.de</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2083,7 +2080,7 @@
         <v>https://www.auto-ankauf-bielefeld.de</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2128,7 +2125,7 @@
         <v>https://www.cuxhaven-autoankauf.de</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2191,7 +2188,7 @@
         <v>https://www.auto-ankauf-gelsenkirchen24.de</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2200,7 +2197,7 @@
         <v>https://www.kfz-ankauf-herne.de</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2209,7 +2206,7 @@
         <v>https://www.kfz-ankauf-bochum.de</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2218,7 +2215,7 @@
         <v>https://www.castrop-rauxel-autoankauf.de</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2227,7 +2224,7 @@
         <v>https://www.auto-ankauf-witten.de</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2236,7 +2233,7 @@
         <v>https://www.auto-ankauf-gladbeck.de</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2245,7 +2242,7 @@
         <v>https://www.autoduisburg.de</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2254,7 +2251,7 @@
         <v>https://www.xn--kfz-ankauf-mnster-e3b.de</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2263,7 +2260,7 @@
         <v>https://www.auto-ankauf-wesel.de</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2281,7 +2278,7 @@
         <v>https://www.autohaan.de</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2290,7 +2287,7 @@
         <v>https://www.unna-auto-ankauf.de</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2299,7 +2296,7 @@
         <v>https://www.solingen-auto.de</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2308,7 +2305,7 @@
         <v>https://www.wermelskirchen-autoankauf.de</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2317,7 +2314,7 @@
         <v>https://www.autohilden.de</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2326,7 +2323,7 @@
         <v>https://www.auto-ankauf-krefeld24.de</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2335,7 +2332,7 @@
         <v>https://www.auto-ankauf-kempen.de</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2353,7 +2350,7 @@
         <v>https://www.autoleverkusen.de</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2371,7 +2368,7 @@
         <v>https://www.xn--mnster-auto-ankauf-m6b.de</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2380,7 +2377,7 @@
         <v>https://www.arnsberg-autoankauf.de</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2389,7 +2386,7 @@
         <v>https://www.auto-ankauf-siegburg.de</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2398,7 +2395,7 @@
         <v>https://www.wiesbaden-auto-ankauf.de</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2407,7 +2404,7 @@
         <v>https://www.frankfurt-am-main-autoankauf.de</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2416,7 +2413,7 @@
         <v>https://www.maintal-autoankauf.de</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2425,7 +2422,7 @@
         <v>https://www.autoankauf-dietzenbach.de</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2443,7 +2440,7 @@
         <v>https://www.autoankauf-griesheim.de</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2452,7 +2449,7 @@
         <v>https://www.xn--kfz-ankauf-wrzburg-x6b.de</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2560,7 +2557,7 @@
         <v>https://www.autoankauf-dillenburg.de</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2569,7 +2566,7 @@
         <v>https://www.kfz-ankauf-marburg.de</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2587,7 +2584,7 @@
         <v>https://www.autoankauf-bad-wildungen.de</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2596,7 +2593,7 @@
         <v>https://www.autoankauf-fritzlar.de</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2605,7 +2602,7 @@
         <v>https://www.auto-ankauf-butzbach.de</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2614,7 +2611,7 @@
         <v>https://www.gebrauchtwagen-ankauf-kassel.de</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2623,7 +2620,7 @@
         <v>https://www.autoankauf-homberg.de</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2632,7 +2629,7 @@
         <v>https://www.autoankauf-hungen.de</v>
       </c>
       <c r="B118" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2668,7 +2665,7 @@
         <v>https://www.auto-ankauf-ahaus.de</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2677,7 +2674,7 @@
         <v>https://www.kfz-ankauf-nettetal.de</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2686,7 +2683,7 @@
         <v>https://www.auto-ankauf-soest.de</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2695,7 +2692,7 @@
         <v>https://www.auto-ankauf-steinfurt.de</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2704,7 +2701,7 @@
         <v>https://www.kleve-auto-ankauf.de</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2713,7 +2710,7 @@
         <v>https://www.autoratingen.de</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2722,7 +2719,7 @@
         <v>https://www.auto-ankauf-lippstadt.de</v>
       </c>
       <c r="B128" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2731,7 +2728,7 @@
         <v>https://www.autoankauf-northeim.de</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2740,7 +2737,7 @@
         <v>https://www.gebrauchtwagen-ankauf-hannover.de</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2749,7 +2746,7 @@
         <v>https://www.autoankauf-duderstadt.de</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2758,7 +2755,7 @@
         <v>https://www.autoankauf-osterholz-scharmbeck.de</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2767,7 +2764,7 @@
         <v>https://www.salzgitter-autoankauf.de</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2776,7 +2773,7 @@
         <v>https://www.autoankauf-wittmund.de</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2785,7 +2782,7 @@
         <v>https://www.autoankauf-peine.de</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2794,7 +2791,7 @@
         <v>https://www.auto-ankauf-rheine.de</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2803,7 +2800,7 @@
         <v>https://www.autobonn.de</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2812,7 +2809,7 @@
         <v>https://www.auto-ankauf-heinsberg.de</v>
       </c>
       <c r="B138" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2821,7 +2818,7 @@
         <v>https://www.autoankauf-brilon.de</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2830,7 +2827,7 @@
         <v>https://www.kfz-ankauf-bielefeld.de</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2839,7 +2836,7 @@
         <v>https://www.gebrauchtwagen-ankauf-paderborn.de</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2848,7 +2845,7 @@
         <v>https://www.auto-ankauf-herford.de</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2866,7 +2863,7 @@
         <v>https://www.auto-ankauf-minden.de</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2875,7 +2872,7 @@
         <v>https://www.auto-ankauf-altenkirchen.de</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2884,7 +2881,7 @@
         <v>https://www.auto-ankauf-neuwied.de</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2893,7 +2890,7 @@
         <v>https://www.montabaur-autoankauf.de</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -2902,7 +2899,7 @@
         <v>https://www.mayen-autoankauf.de</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2911,7 +2908,7 @@
         <v>https://www.gotha-autoankauf.de</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2920,7 +2917,7 @@
         <v>https://www.nordhausen-auto-ankauf.de</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2929,7 +2926,7 @@
         <v>https://www.autoankauf-speyer.de</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2938,7 +2935,7 @@
         <v>https://www.autoankauf-wittlich.de</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2947,7 +2944,7 @@
         <v>https://www.kfz-ankauf-trier.de</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2956,7 +2953,7 @@
         <v>https://www.autoankauf-pforzheim.de</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2965,7 +2962,7 @@
         <v>https://www.gebrauchtwagen-ankauf-heilbronn.de</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2983,7 +2980,7 @@
         <v>https://www.wolfsburg-autoankauf.de</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -2992,7 +2989,7 @@
         <v>https://www.autoankauf-merzig.de</v>
       </c>
       <c r="B158" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3019,7 +3016,7 @@
         <v>https://www.gebrauchtwagen-ankauf-mainz.de</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3028,7 +3025,7 @@
         <v>https://www.autoankauf-gerolstein.de</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3037,7 +3034,7 @@
         <v>https://www.auto-ankauf-daun.de</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3082,7 +3079,7 @@
         <v>https://www.kfz-ankauf-mainz.de</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3091,7 +3088,7 @@
         <v>https://www.autoankauf-wernigerode.de</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3109,7 +3106,7 @@
         <v>https://www.autoankauf-bad-kissingen.de</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3118,7 +3115,7 @@
         <v>https://www.xn--saarbrcken-gebrauchtwagenankauf-tid.de</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3127,7 +3124,7 @@
         <v>https://www.auto-ankauf-miltenberg.de</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.3">
@@ -3136,7 +3133,7 @@
         <v>https://www.schweinfurt-auto-ankauf.de</v>
       </c>
       <c r="B174" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3163,7 +3160,7 @@
         <v>https://www.autoankauf-sinsheim.de</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3181,7 +3178,7 @@
         <v>https://www.auto-ankauf-eppingen.de</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3190,7 +3187,7 @@
         <v>https://www.auto-ankauf-karlsruhe.de</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3199,7 +3196,7 @@
         <v>https://www.autoankauf-karlsbad.de</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="182" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3208,7 +3205,7 @@
         <v>https://www.autoankauf-mosbach.de</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3217,7 +3214,7 @@
         <v>https://www.auto-ankauf-magdeburg.de</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="184" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3226,7 +3223,7 @@
         <v>https://www.auto-ankauf-bamberg.de</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="185" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3235,7 +3232,7 @@
         <v>https://www.auto-ankauf-ludwigsburg.de</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="186" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3253,7 +3250,7 @@
         <v>https://www.halle-auto-ankauf.de</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3262,7 +3259,7 @@
         <v>https://www.autoankauf-halle-saale.de</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="189" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3271,7 +3268,7 @@
         <v>https://www.gebrauchtwagen-ankauf-stuttgart.de</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="190" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3280,7 +3277,7 @@
         <v>https://www.stuttgart-auto-ankauf.de</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="191" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3298,16 +3295,16 @@
         <v>https://www.autoankauf-bad-segeberg.de</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="193" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A193" t="str">
-        <f t="shared" ref="A193:A256" si="5">"https://www." &amp; B193</f>
+        <f t="shared" ref="A193:A255" si="5">"https://www." &amp; B193</f>
         <v>https://www.autoankauf-offenburg.de</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3316,7 +3313,7 @@
         <v>https://www.auto-ankauf-forchheim.de</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3334,7 +3331,7 @@
         <v>https://www.herrenberg-autoankauf.de</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="197" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3343,7 +3340,7 @@
         <v>https://www.xn--autoankauf-tbingen-x6b.de</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="198" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3352,7 +3349,7 @@
         <v>https://www.kfz-ankauf-reutlingen.de</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="199" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3361,7 +3358,7 @@
         <v>https://www.xn--autoankauf-gppingen-16b.de</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="200" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3370,7 +3367,7 @@
         <v>https://www.xn--kfz-ankauf-nrnberg-x6b.de</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="201" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3379,7 +3376,7 @@
         <v>https://www.auto-ankauf-aalen.de</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="202" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3388,7 +3385,7 @@
         <v>https://www.leipzig-autoankauf.de</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="203" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3397,7 +3394,7 @@
         <v>https://www.autoankauf-schleswig.de</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="204" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3406,7 +3403,7 @@
         <v>https://www.autoankauf-preetz.de</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="205" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3415,7 +3412,7 @@
         <v>https://www.autoankauf-schwabach.de</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="206" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3424,7 +3421,7 @@
         <v>https://www.autoankauf-altenburg.de</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3433,7 +3430,7 @@
         <v>https://www.autoankauf-zwickau.de</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="208" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3442,7 +3439,7 @@
         <v>https://www.freiburg-auto-ankauf.de</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3451,7 +3448,7 @@
         <v>https://www.gebrauchtwagen-ankauf-ulm.de</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="210" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3460,7 +3457,7 @@
         <v>https://www.kfz-ankauf-dresden.de</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3478,7 +3475,7 @@
         <v>https://www.kfz-ankauf-regensburg.de</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3487,7 +3484,7 @@
         <v>https://www.auto-ankauf-memmingen.de</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3496,7 +3493,7 @@
         <v>https://www.auto-ankauf-ravensburg.de</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3505,7 +3502,7 @@
         <v>https://www.autoankauf-pfaffenhofen.de</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3514,7 +3511,7 @@
         <v>https://www.autoankauf-konstanz.de</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3523,7 +3520,7 @@
         <v>https://www.auto-ankauf-konstanz.de</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3532,7 +3529,7 @@
         <v>https://www.auto-ankauf-amberg.de</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -3547,106 +3544,106 @@
     <row r="220" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A220" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoankauf-mainburg.de</v>
+        <v>https://www.auto-ankauf-dachau.de</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A221" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.auto-ankauf-dachau.de</v>
+        <v>https://www.auto-ankauf-landshut.de</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A222" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.auto-ankauf-landshut.de</v>
+        <v>https://www.xn--mnchen-auto-ankauf-m6b.de</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>130</v>
+        <v>192</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A223" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.xn--mnchen-auto-ankauf-m6b.de</v>
+        <v>https://www.autoankauf-bautzen.de</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>193</v>
+        <v>117</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A224" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoankauf-bautzen.de</v>
+        <v>https://www.auto-ankauf-deggendorf.de</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A225" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.auto-ankauf-deggendorf.de</v>
+        <v>https://www.autoankauf-murnau.de</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>150</v>
+        <v>115</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A226" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoankauf-murnau.de</v>
+        <v>https://www.autoankauf-pfarrkirchen.de</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>116</v>
+        <v>63</v>
       </c>
     </row>
     <row r="227" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A227" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoankauf-pfarrkirchen.de</v>
+        <v>https://www.auto-ankauf-passau.de</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
     </row>
     <row r="228" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A228" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.auto-ankauf-passau.de</v>
+        <v>https://www.auto-ankauf-traunstein.de</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>88</v>
+        <v>141</v>
       </c>
     </row>
     <row r="229" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A229" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.auto-ankauf-traunstein.de</v>
+        <v>https://www.autoankauf-siegsdorf.de</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A230" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoankauf-siegsdorf.de</v>
-      </c>
-      <c r="B230" s="2" t="s">
-        <v>62</v>
+        <v>https://www.leverkusen-schrott.de</v>
+      </c>
+      <c r="B230" s="4" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A231" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.leverkusen-schrott.de</v>
+        <v>https://www.schrott-ankauf-bonn.de</v>
       </c>
       <c r="B231" s="4" t="s">
         <v>207</v>
@@ -3655,7 +3652,7 @@
     <row r="232" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A232" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrott-ankauf-bonn.de</v>
+        <v>https://www.schrott-ankauf-duisburg.de</v>
       </c>
       <c r="B232" s="4" t="s">
         <v>208</v>
@@ -3664,7 +3661,7 @@
     <row r="233" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A233" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrott-ankauf-duisburg.de</v>
+        <v>https://www.schrott-ankauf-essen.de</v>
       </c>
       <c r="B233" s="4" t="s">
         <v>209</v>
@@ -3673,7 +3670,7 @@
     <row r="234" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A234" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrott-ankauf-essen.de</v>
+        <v>https://www.schrott-ankauf-gelsenkirchen.de</v>
       </c>
       <c r="B234" s="4" t="s">
         <v>210</v>
@@ -3682,7 +3679,7 @@
     <row r="235" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A235" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrott-ankauf-gelsenkirchen.de</v>
+        <v>https://www.schrott-ankauf-wuppertal.de</v>
       </c>
       <c r="B235" s="4" t="s">
         <v>211</v>
@@ -3691,7 +3688,7 @@
     <row r="236" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A236" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrott-ankauf-wuppertal.de</v>
+        <v>https://www.schrott-recklinghausen.de</v>
       </c>
       <c r="B236" s="4" t="s">
         <v>212</v>
@@ -3700,7 +3697,7 @@
     <row r="237" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A237" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrott-recklinghausen.de</v>
+        <v>https://www.schrottgummersbach.de</v>
       </c>
       <c r="B237" s="4" t="s">
         <v>213</v>
@@ -3709,7 +3706,7 @@
     <row r="238" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A238" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrottgummersbach.de</v>
+        <v>https://www.schrottlohmar.de</v>
       </c>
       <c r="B238" s="4" t="s">
         <v>214</v>
@@ -3718,7 +3715,7 @@
     <row r="239" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A239" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrottlohmar.de</v>
+        <v>https://www.schrottolpe.de</v>
       </c>
       <c r="B239" s="4" t="s">
         <v>215</v>
@@ -3727,7 +3724,7 @@
     <row r="240" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A240" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrottolpe.de</v>
+        <v>https://www.schrottratingen.de</v>
       </c>
       <c r="B240" s="4" t="s">
         <v>216</v>
@@ -3736,7 +3733,7 @@
     <row r="241" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A241" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrottratingen.de</v>
+        <v>https://www.schrottsiegburg.de</v>
       </c>
       <c r="B241" s="4" t="s">
         <v>217</v>
@@ -3745,7 +3742,7 @@
     <row r="242" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A242" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrottsiegburg.de</v>
+        <v>https://www.schrottunna.de</v>
       </c>
       <c r="B242" s="4" t="s">
         <v>218</v>
@@ -3754,16 +3751,16 @@
     <row r="243" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A243" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.schrottunna.de</v>
-      </c>
-      <c r="B243" s="4" t="s">
-        <v>219</v>
+        <v>https://www.ahrensburg-autoverwertung.de</v>
+      </c>
+      <c r="B243" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A244" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.ahrensburg-autoverwertung.de</v>
+        <v>https://www.autoverwertung-bergischgladbach.de</v>
       </c>
       <c r="B244" t="s">
         <v>243</v>
@@ -3772,7 +3769,7 @@
     <row r="245" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A245" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-bergischgladbach.de</v>
+        <v>https://www.autoverwertung-dithmarschen.de</v>
       </c>
       <c r="B245" t="s">
         <v>244</v>
@@ -3781,7 +3778,7 @@
     <row r="246" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A246" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-dithmarschen.de</v>
+        <v>https://www.autoverwertung-dormagen.de</v>
       </c>
       <c r="B246" t="s">
         <v>245</v>
@@ -3790,7 +3787,7 @@
     <row r="247" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A247" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-dormagen.de</v>
+        <v>https://www.autoverwertung-elmshorn.de</v>
       </c>
       <c r="B247" t="s">
         <v>246</v>
@@ -3799,7 +3796,7 @@
     <row r="248" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A248" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-elmshorn.de</v>
+        <v>https://www.autoverwertung-geesthacht.de</v>
       </c>
       <c r="B248" t="s">
         <v>247</v>
@@ -3808,7 +3805,7 @@
     <row r="249" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A249" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-geesthacht.de</v>
+        <v>https://www.autoverwertung-glinde.de</v>
       </c>
       <c r="B249" t="s">
         <v>248</v>
@@ -3817,7 +3814,7 @@
     <row r="250" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A250" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-glinde.de</v>
+        <v>https://www.autoverwertung-göttingen.de</v>
       </c>
       <c r="B250" t="s">
         <v>249</v>
@@ -3826,7 +3823,7 @@
     <row r="251" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A251" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-göttingen.de</v>
+        <v>https://www.autoverwertung-grevenbroich.de</v>
       </c>
       <c r="B251" t="s">
         <v>250</v>
@@ -3835,7 +3832,7 @@
     <row r="252" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A252" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-grevenbroich.de</v>
+        <v>https://www.autoverwertung-iserlohn.de</v>
       </c>
       <c r="B252" t="s">
         <v>251</v>
@@ -3844,7 +3841,7 @@
     <row r="253" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A253" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-iserlohn.de</v>
+        <v>https://www.autoverwertung-itzehoe.de</v>
       </c>
       <c r="B253" t="s">
         <v>252</v>
@@ -3853,7 +3850,7 @@
     <row r="254" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A254" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-itzehoe.de</v>
+        <v>https://www.autoverwertung-kassel.de</v>
       </c>
       <c r="B254" t="s">
         <v>253</v>
@@ -3862,7 +3859,7 @@
     <row r="255" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A255" t="str">
         <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-kassel.de</v>
+        <v>https://www.autoverwertung-kreuztal.de</v>
       </c>
       <c r="B255" t="s">
         <v>254</v>
@@ -3870,8 +3867,8 @@
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A256" t="str">
-        <f t="shared" si="5"/>
-        <v>https://www.autoverwertung-kreuztal.de</v>
+        <f t="shared" ref="A256:A319" si="6">"https://www." &amp; B256</f>
+        <v>https://www.autoverwertung-leverkusen.de</v>
       </c>
       <c r="B256" t="s">
         <v>255</v>
@@ -3879,8 +3876,8 @@
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A257" t="str">
-        <f t="shared" ref="A257:A320" si="6">"https://www." &amp; B257</f>
-        <v>https://www.autoverwertung-leverkusen.de</v>
+        <f t="shared" si="6"/>
+        <v>https://www.autoverwertung-lohmar.de</v>
       </c>
       <c r="B257" t="s">
         <v>256</v>
@@ -3889,7 +3886,7 @@
     <row r="258" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A258" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-lohmar.de</v>
+        <v>https://www.autoverwertung-lübeck.de</v>
       </c>
       <c r="B258" t="s">
         <v>257</v>
@@ -3898,7 +3895,7 @@
     <row r="259" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A259" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-lübeck.de</v>
+        <v>https://www.autoverwertung-lüdenscheid.de</v>
       </c>
       <c r="B259" t="s">
         <v>258</v>
@@ -3907,7 +3904,7 @@
     <row r="260" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A260" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-lüdenscheid.de</v>
+        <v>https://www.autoverwertung-marl.de</v>
       </c>
       <c r="B260" t="s">
         <v>259</v>
@@ -3916,7 +3913,7 @@
     <row r="261" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A261" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-marl.de</v>
+        <v>https://www.autoverwertung-moers.de</v>
       </c>
       <c r="B261" t="s">
         <v>260</v>
@@ -3925,7 +3922,7 @@
     <row r="262" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A262" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-moers.de</v>
+        <v>https://www.autoverwertung-neumünster.de</v>
       </c>
       <c r="B262" t="s">
         <v>261</v>
@@ -3934,7 +3931,7 @@
     <row r="263" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A263" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-neumünster.de</v>
+        <v>https://www.autoverwertung-nordfriesland.de</v>
       </c>
       <c r="B263" t="s">
         <v>262</v>
@@ -3943,7 +3940,7 @@
     <row r="264" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A264" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-nordfriesland.de</v>
+        <v>https://www.olpe-autoentsorgung.de</v>
       </c>
       <c r="B264" t="s">
         <v>263</v>
@@ -3952,7 +3949,7 @@
     <row r="265" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A265" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.olpe-autoentsorgung.de</v>
+        <v>https://www.autoverwertung-ostholstein.de</v>
       </c>
       <c r="B265" t="s">
         <v>264</v>
@@ -3961,7 +3958,7 @@
     <row r="266" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A266" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-ostholstein.de</v>
+        <v>https://www.autoverwertung-pinneberg.de</v>
       </c>
       <c r="B266" t="s">
         <v>265</v>
@@ -3970,7 +3967,7 @@
     <row r="267" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A267" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-pinneberg.de</v>
+        <v>https://www.autoverwertung-plön.de</v>
       </c>
       <c r="B267" t="s">
         <v>266</v>
@@ -3979,7 +3976,7 @@
     <row r="268" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A268" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-plön.de</v>
+        <v>https://www.autoverwertung-ratingen.de</v>
       </c>
       <c r="B268" t="s">
         <v>267</v>
@@ -3988,7 +3985,7 @@
     <row r="269" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A269" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-ratingen.de</v>
+        <v>https://www.autoverwertung-remscheid.de</v>
       </c>
       <c r="B269" t="s">
         <v>268</v>
@@ -3997,7 +3994,7 @@
     <row r="270" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A270" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-remscheid.de</v>
+        <v>https://www.autoverwertung-rendsburg.de</v>
       </c>
       <c r="B270" t="s">
         <v>269</v>
@@ -4006,7 +4003,7 @@
     <row r="271" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A271" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-rendsburg.de</v>
+        <v>https://www.autoverwertung-segeberg.de</v>
       </c>
       <c r="B271" t="s">
         <v>270</v>
@@ -4015,7 +4012,7 @@
     <row r="272" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A272" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-segeberg.de</v>
+        <v>https://www.autoverwertung-siegburg.de</v>
       </c>
       <c r="B272" t="s">
         <v>271</v>
@@ -4024,7 +4021,7 @@
     <row r="273" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A273" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-siegburg.de</v>
+        <v>https://www.autoverwertung-solingen.de</v>
       </c>
       <c r="B273" t="s">
         <v>272</v>
@@ -4033,7 +4030,7 @@
     <row r="274" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A274" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-solingen.de</v>
+        <v>https://www.autoverwertung-steinburg.de</v>
       </c>
       <c r="B274" t="s">
         <v>273</v>
@@ -4042,7 +4039,7 @@
     <row r="275" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A275" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-steinburg.de</v>
+        <v>https://www.autoverwertung-stormarn.de</v>
       </c>
       <c r="B275" t="s">
         <v>274</v>
@@ -4051,7 +4048,7 @@
     <row r="276" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A276" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-stormarn.de</v>
+        <v>https://www.autoverwertung-viersen.de</v>
       </c>
       <c r="B276" t="s">
         <v>275</v>
@@ -4060,7 +4057,7 @@
     <row r="277" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A277" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-viersen.de</v>
+        <v>https://www.autoverwertung-wedel.de</v>
       </c>
       <c r="B277" t="s">
         <v>276</v>
@@ -4069,7 +4066,7 @@
     <row r="278" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A278" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-wedel.de</v>
+        <v>https://www.autoverwertung-witten.de</v>
       </c>
       <c r="B278" t="s">
         <v>277</v>
@@ -4078,7 +4075,7 @@
     <row r="279" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A279" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwertung-witten.de</v>
+        <v>https://www.bergkamen-autoverwertung.de</v>
       </c>
       <c r="B279" t="s">
         <v>278</v>
@@ -4087,7 +4084,7 @@
     <row r="280" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A280" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.bergkamen-autoverwertung.de</v>
+        <v>https://www.bonn-autoverwertung.de</v>
       </c>
       <c r="B280" t="s">
         <v>279</v>
@@ -4096,7 +4093,7 @@
     <row r="281" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A281" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.bonn-autoverwertung.de</v>
+        <v>https://www.borken-autoverwertung.de</v>
       </c>
       <c r="B281" t="s">
         <v>280</v>
@@ -4105,7 +4102,7 @@
     <row r="282" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A282" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.borken-autoverwertung.de</v>
+        <v>https://www.bremen-autoverwertung.de</v>
       </c>
       <c r="B282" t="s">
         <v>281</v>
@@ -4114,7 +4111,7 @@
     <row r="283" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A283" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.bremen-autoverwertung.de</v>
+        <v>https://www.erkrath-autoverwertung.de</v>
       </c>
       <c r="B283" t="s">
         <v>282</v>
@@ -4123,7 +4120,7 @@
     <row r="284" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A284" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.erkrath-autoverwertung.de</v>
+        <v>https://www.flensburg-autoverwertung.de</v>
       </c>
       <c r="B284" t="s">
         <v>283</v>
@@ -4132,7 +4129,7 @@
     <row r="285" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A285" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.flensburg-autoverwertung.de</v>
+        <v>https://www.gütersloh-autoverwertung.de</v>
       </c>
       <c r="B285" t="s">
         <v>284</v>
@@ -4141,7 +4138,7 @@
     <row r="286" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A286" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.gütersloh-autoverwertung.de</v>
+        <v>https://www.hagen-autoverwertung.de</v>
       </c>
       <c r="B286" t="s">
         <v>285</v>
@@ -4150,7 +4147,7 @@
     <row r="287" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A287" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.hagen-autoverwertung.de</v>
+        <v>https://www.hamburg-autoverschrottung.de</v>
       </c>
       <c r="B287" t="s">
         <v>286</v>
@@ -4159,7 +4156,7 @@
     <row r="288" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A288" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.hamburg-autoverschrottung.de</v>
+        <v>https://www.hamm-autoverwertung.de</v>
       </c>
       <c r="B288" t="s">
         <v>287</v>
@@ -4168,7 +4165,7 @@
     <row r="289" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A289" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.hamm-autoverwertung.de</v>
+        <v>https://www.hannover-autoverwertung.de</v>
       </c>
       <c r="B289" t="s">
         <v>288</v>
@@ -4177,7 +4174,7 @@
     <row r="290" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A290" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.hannover-autoverwertung.de</v>
+        <v>https://www.kiel-autoverwertung.de</v>
       </c>
       <c r="B290" t="s">
         <v>289</v>
@@ -4186,7 +4183,7 @@
     <row r="291" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A291" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.kiel-autoverwertung.de</v>
+        <v>https://www.koblenz-autoverwertung.de</v>
       </c>
       <c r="B291" t="s">
         <v>290</v>
@@ -4195,7 +4192,7 @@
     <row r="292" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A292" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.koblenz-autoverwertung.de</v>
+        <v>https://www.krefeld-autoverwertung.de</v>
       </c>
       <c r="B292" t="s">
         <v>291</v>
@@ -4204,7 +4201,7 @@
     <row r="293" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A293" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.krefeld-autoverwertung.de</v>
+        <v>https://www.mönchengladbach-autoverwertung.de</v>
       </c>
       <c r="B293" t="s">
         <v>292</v>
@@ -4213,7 +4210,7 @@
     <row r="294" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A294" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.mönchengladbach-autoverwertung.de</v>
+        <v>https://www.neuss-autoverwertung.de</v>
       </c>
       <c r="B294" t="s">
         <v>293</v>
@@ -4222,7 +4219,7 @@
     <row r="295" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A295" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.neuss-autoverwertung.de</v>
+        <v>https://www.neuwied-autoverwertung.de</v>
       </c>
       <c r="B295" t="s">
         <v>294</v>
@@ -4231,7 +4228,7 @@
     <row r="296" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A296" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.neuwied-autoverwertung.de</v>
+        <v>https://www.norderstedt-autoverwertung.de</v>
       </c>
       <c r="B296" t="s">
         <v>295</v>
@@ -4240,7 +4237,7 @@
     <row r="297" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A297" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.norderstedt-autoverwertung.de</v>
+        <v>https://www.oberhausen-autoverwertung.de</v>
       </c>
       <c r="B297" t="s">
         <v>296</v>
@@ -4249,7 +4246,7 @@
     <row r="298" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A298" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.oberhausen-autoverwertung.de</v>
+        <v>https://www.oldenburg-autoverwertung.de</v>
       </c>
       <c r="B298" t="s">
         <v>297</v>
@@ -4258,7 +4255,7 @@
     <row r="299" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A299" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.oldenburg-autoverwertung.de</v>
+        <v>https://www.osnabrück-autoverwertung.de</v>
       </c>
       <c r="B299" t="s">
         <v>298</v>
@@ -4267,7 +4264,7 @@
     <row r="300" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A300" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.osnabrück-autoverwertung.de</v>
+        <v>https://www.rheinbach-autoverwertung.de</v>
       </c>
       <c r="B300" t="s">
         <v>299</v>
@@ -4276,7 +4273,7 @@
     <row r="301" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A301" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.rheinbach-autoverwertung.de</v>
+        <v>https://www.schwelm-autoverwertung.de</v>
       </c>
       <c r="B301" t="s">
         <v>300</v>
@@ -4285,7 +4282,7 @@
     <row r="302" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A302" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.schwelm-autoverwertung.de</v>
+        <v>https://www.siegen-autoverwertung.de</v>
       </c>
       <c r="B302" t="s">
         <v>301</v>
@@ -4294,7 +4291,7 @@
     <row r="303" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A303" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.siegen-autoverwertung.de</v>
+        <v>https://www.autoverwerter-aachen.de</v>
       </c>
       <c r="B303" t="s">
         <v>302</v>
@@ -4303,7 +4300,7 @@
     <row r="304" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A304" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-aachen.de</v>
+        <v>https://www.autoverwerter-ahlen.de</v>
       </c>
       <c r="B304" t="s">
         <v>303</v>
@@ -4312,7 +4309,7 @@
     <row r="305" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A305" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-ahlen.de</v>
+        <v>https://www.autoverwerter-alzey.de</v>
       </c>
       <c r="B305" t="s">
         <v>304</v>
@@ -4321,7 +4318,7 @@
     <row r="306" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A306" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-alzey.de</v>
+        <v>https://www.autoverwerter-bocholt.de</v>
       </c>
       <c r="B306" t="s">
         <v>305</v>
@@ -4330,7 +4327,7 @@
     <row r="307" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A307" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-bocholt.de</v>
+        <v>https://www.autoverwerter-borken.de</v>
       </c>
       <c r="B307" t="s">
         <v>306</v>
@@ -4339,7 +4336,7 @@
     <row r="308" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A308" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-borken.de</v>
+        <v>https://www.autoverwerter-bramsche.de</v>
       </c>
       <c r="B308" t="s">
         <v>307</v>
@@ -4348,7 +4345,7 @@
     <row r="309" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A309" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-bramsche.de</v>
+        <v>https://www.autoverwerter-delmenhorst.de</v>
       </c>
       <c r="B309" t="s">
         <v>308</v>
@@ -4357,7 +4354,7 @@
     <row r="310" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A310" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-delmenhorst.de</v>
+        <v>https://www.autoverwerter-dorsten.de</v>
       </c>
       <c r="B310" t="s">
         <v>309</v>
@@ -4366,7 +4363,7 @@
     <row r="311" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A311" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-dorsten.de</v>
+        <v>https://www.autoverwerter-frechen.de</v>
       </c>
       <c r="B311" t="s">
         <v>310</v>
@@ -4375,7 +4372,7 @@
     <row r="312" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A312" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-frechen.de</v>
+        <v>https://www.autoverwerter-geestland.de</v>
       </c>
       <c r="B312" t="s">
         <v>311</v>
@@ -4384,7 +4381,7 @@
     <row r="313" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A313" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-geestland.de</v>
+        <v>https://www.autoverwerter-germersheim.de</v>
       </c>
       <c r="B313" t="s">
         <v>312</v>
@@ -4393,7 +4390,7 @@
     <row r="314" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A314" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-germersheim.de</v>
+        <v>https://www.autoverwerter-gladbeck.de</v>
       </c>
       <c r="B314" t="s">
         <v>313</v>
@@ -4402,7 +4399,7 @@
     <row r="315" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A315" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-gladbeck.de</v>
+        <v>https://www.autoverwerter-heiligenhaus.de</v>
       </c>
       <c r="B315" t="s">
         <v>314</v>
@@ -4411,7 +4408,7 @@
     <row r="316" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A316" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-heiligenhaus.de</v>
+        <v>https://www.autoverwerter-herne.de</v>
       </c>
       <c r="B316" t="s">
         <v>315</v>
@@ -4420,7 +4417,7 @@
     <row r="317" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A317" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-herne.de</v>
+        <v>https://www.autoverwerter-hildesheim.de</v>
       </c>
       <c r="B317" t="s">
         <v>316</v>
@@ -4429,7 +4426,7 @@
     <row r="318" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A318" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-hildesheim.de</v>
+        <v>https://www.autoverwerter-kaiserslautern.de</v>
       </c>
       <c r="B318" t="s">
         <v>317</v>
@@ -4438,7 +4435,7 @@
     <row r="319" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A319" t="str">
         <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-kaiserslautern.de</v>
+        <v>https://www.autoverwerter-kamen.de</v>
       </c>
       <c r="B319" t="s">
         <v>318</v>
@@ -4446,8 +4443,8 @@
     </row>
     <row r="320" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A320" t="str">
-        <f t="shared" si="6"/>
-        <v>https://www.autoverwerter-kamen.de</v>
+        <f t="shared" ref="A320:A362" si="7">"https://www." &amp; B320</f>
+        <v>https://www.autoverwerter-kleve.de</v>
       </c>
       <c r="B320" t="s">
         <v>319</v>
@@ -4455,8 +4452,8 @@
     </row>
     <row r="321" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A321" t="str">
-        <f t="shared" ref="A321:A363" si="7">"https://www." &amp; B321</f>
-        <v>https://www.autoverwerter-kleve.de</v>
+        <f t="shared" si="7"/>
+        <v>https://www.autoverwerter-lahnstein.de</v>
       </c>
       <c r="B321" t="s">
         <v>320</v>
@@ -4465,7 +4462,7 @@
     <row r="322" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A322" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-lahnstein.de</v>
+        <v>https://www.autoverwerter-mayen.de</v>
       </c>
       <c r="B322" t="s">
         <v>321</v>
@@ -4474,7 +4471,7 @@
     <row r="323" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A323" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-mayen.de</v>
+        <v>https://www.autoverwerter-meerbusch.de</v>
       </c>
       <c r="B323" t="s">
         <v>322</v>
@@ -4483,7 +4480,7 @@
     <row r="324" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A324" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-meerbusch.de</v>
+        <v>https://www.autoverwerter-meppen.de</v>
       </c>
       <c r="B324" t="s">
         <v>323</v>
@@ -4492,7 +4489,7 @@
     <row r="325" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A325" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-meppen.de</v>
+        <v>https://www.autoverwerter-nettetal.de</v>
       </c>
       <c r="B325" t="s">
         <v>324</v>
@@ -4501,7 +4498,7 @@
     <row r="326" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A326" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-nettetal.de</v>
+        <v>https://www.autoverwerter-paderborn.de</v>
       </c>
       <c r="B326" t="s">
         <v>325</v>
@@ -4510,7 +4507,7 @@
     <row r="327" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A327" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-paderborn.de</v>
+        <v>https://www.autoverwerter-pirmasens.de</v>
       </c>
       <c r="B327" t="s">
         <v>326</v>
@@ -4519,7 +4516,7 @@
     <row r="328" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A328" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-pirmasens.de</v>
+        <v>https://www.autoverwerter-salzgitter.de</v>
       </c>
       <c r="B328" t="s">
         <v>327</v>
@@ -4528,7 +4525,7 @@
     <row r="329" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A329" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-salzgitter.de</v>
+        <v>https://www.autoverwerter-schifferstadt.de</v>
       </c>
       <c r="B329" t="s">
         <v>328</v>
@@ -4537,7 +4534,7 @@
     <row r="330" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A330" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-schifferstadt.de</v>
+        <v>https://www.autoverwerter-schwerte.de</v>
       </c>
       <c r="B330" t="s">
         <v>329</v>
@@ -4546,7 +4543,7 @@
     <row r="331" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A331" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-schwerte.de</v>
+        <v>https://www.autoverwerter-stade.de</v>
       </c>
       <c r="B331" t="s">
         <v>330</v>
@@ -4555,7 +4552,7 @@
     <row r="332" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A332" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-stade.de</v>
+        <v>https://www.autoverwerter-wilhelmshaven.de</v>
       </c>
       <c r="B332" t="s">
         <v>331</v>
@@ -4564,7 +4561,7 @@
     <row r="333" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A333" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-wilhelmshaven.de</v>
+        <v>https://www.autoverwerter-wittlich.de</v>
       </c>
       <c r="B333" t="s">
         <v>332</v>
@@ -4573,7 +4570,7 @@
     <row r="334" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A334" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-wittlich.de</v>
+        <v>https://www.autoverwerter-würzburg.de</v>
       </c>
       <c r="B334" t="s">
         <v>333</v>
@@ -4582,7 +4579,7 @@
     <row r="335" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A335" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwerter-würzburg.de</v>
+        <v>https://www.autoverwertung-baesweiler.de</v>
       </c>
       <c r="B335" t="s">
         <v>334</v>
@@ -4591,7 +4588,7 @@
     <row r="336" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A336" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-baesweiler.de</v>
+        <v>https://www.autoverwertung-bornheim.de</v>
       </c>
       <c r="B336" t="s">
         <v>335</v>
@@ -4600,7 +4597,7 @@
     <row r="337" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A337" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-bornheim.de</v>
+        <v>https://www.autoverwertung-burgdorf.de</v>
       </c>
       <c r="B337" t="s">
         <v>336</v>
@@ -4609,7 +4606,7 @@
     <row r="338" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A338" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-burgdorf.de</v>
+        <v>https://www.autoverwertung-einbeck.de</v>
       </c>
       <c r="B338" t="s">
         <v>337</v>
@@ -4618,7 +4615,7 @@
     <row r="339" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A339" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-einbeck.de</v>
+        <v>https://www.autoverwertung-erftstadt.de</v>
       </c>
       <c r="B339" t="s">
         <v>338</v>
@@ -4627,7 +4624,7 @@
     <row r="340" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A340" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-erftstadt.de</v>
+        <v>https://www.autoverwertung-eschborn.de</v>
       </c>
       <c r="B340" t="s">
         <v>339</v>
@@ -4636,7 +4633,7 @@
     <row r="341" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A341" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-eschborn.de</v>
+        <v>https://www.autoverwertung-espelkamp.de</v>
       </c>
       <c r="B341" t="s">
         <v>340</v>
@@ -4645,7 +4642,7 @@
     <row r="342" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A342" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-espelkamp.de</v>
+        <v>https://www.autoverwertung-gifhorn.de</v>
       </c>
       <c r="B342" t="s">
         <v>341</v>
@@ -4654,7 +4651,7 @@
     <row r="343" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A343" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-gifhorn.de</v>
+        <v>https://www.autoverwertung-goch.de</v>
       </c>
       <c r="B343" t="s">
         <v>342</v>
@@ -4663,7 +4660,7 @@
     <row r="344" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A344" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-goch.de</v>
+        <v>https://www.autoverwertung-hofgeismar.de</v>
       </c>
       <c r="B344" t="s">
         <v>343</v>
@@ -4672,7 +4669,7 @@
     <row r="345" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A345" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-hofgeismar.de</v>
+        <v>https://www.autoverwertung-idstein.de</v>
       </c>
       <c r="B345" t="s">
         <v>344</v>
@@ -4681,7 +4678,7 @@
     <row r="346" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A346" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-idstein.de</v>
+        <v>https://www.autoverwertung-kelkheim.de</v>
       </c>
       <c r="B346" t="s">
         <v>345</v>
@@ -4690,7 +4687,7 @@
     <row r="347" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A347" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-kelkheim.de</v>
+        <v>https://www.autoverwertung-langenfeld.de</v>
       </c>
       <c r="B347" t="s">
         <v>346</v>
@@ -4699,7 +4696,7 @@
     <row r="348" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A348" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-langenfeld.de</v>
+        <v>https://www.autoverwertung-lemgo.de</v>
       </c>
       <c r="B348" t="s">
         <v>347</v>
@@ -4708,7 +4705,7 @@
     <row r="349" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A349" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-lemgo.de</v>
+        <v>https://www.autoverwertung-lippstadt.de</v>
       </c>
       <c r="B349" t="s">
         <v>348</v>
@@ -4717,7 +4714,7 @@
     <row r="350" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A350" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-lippstadt.de</v>
+        <v>https://www.autoverwertung-mülheim.de</v>
       </c>
       <c r="B350" t="s">
         <v>349</v>
@@ -4726,7 +4723,7 @@
     <row r="351" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A351" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-mülheim.de</v>
+        <v>https://www.autoverwertung-overath.de</v>
       </c>
       <c r="B351" t="s">
         <v>350</v>
@@ -4735,7 +4732,7 @@
     <row r="352" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A352" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-overath.de</v>
+        <v>https://www.autoverwertung-raesfeld.de</v>
       </c>
       <c r="B352" t="s">
         <v>351</v>
@@ -4744,7 +4741,7 @@
     <row r="353" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A353" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-raesfeld.de</v>
+        <v>https://www.autoverwertung-salzkotten.de</v>
       </c>
       <c r="B353" t="s">
         <v>352</v>
@@ -4753,7 +4750,7 @@
     <row r="354" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A354" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-salzkotten.de</v>
+        <v>https://www.autoverwertung-salzwedel.de</v>
       </c>
       <c r="B354" t="s">
         <v>353</v>
@@ -4762,7 +4759,7 @@
     <row r="355" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A355" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-salzwedel.de</v>
+        <v>https://www.autoverwertung-uelzen.de</v>
       </c>
       <c r="B355" t="s">
         <v>354</v>
@@ -4771,7 +4768,7 @@
     <row r="356" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A356" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-uelzen.de</v>
+        <v>https://www.autoverwertung-vreden.de</v>
       </c>
       <c r="B356" t="s">
         <v>355</v>
@@ -4780,7 +4777,7 @@
     <row r="357" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A357" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-vreden.de</v>
+        <v>https://www.autoverwertung-walsrode.de</v>
       </c>
       <c r="B357" t="s">
         <v>356</v>
@@ -4789,7 +4786,7 @@
     <row r="358" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A358" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-walsrode.de</v>
+        <v>https://www.autoverwertung-wetter.de</v>
       </c>
       <c r="B358" t="s">
         <v>357</v>
@@ -4798,7 +4795,7 @@
     <row r="359" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A359" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.autoverwertung-wetter.de</v>
+        <v>https://www.köln-autoverwertung.de</v>
       </c>
       <c r="B359" t="s">
         <v>358</v>
@@ -4807,7 +4804,7 @@
     <row r="360" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A360" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.köln-autoverwertung.de</v>
+        <v>https://www.stuttgart-autoverwertung.de</v>
       </c>
       <c r="B360" t="s">
         <v>359</v>
@@ -4816,7 +4813,7 @@
     <row r="361" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A361" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.stuttgart-autoverwertung.de</v>
+        <v>https://www.velbert-autoverwertung.de</v>
       </c>
       <c r="B361" t="s">
         <v>360</v>
@@ -4825,19 +4822,10 @@
     <row r="362" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A362" t="str">
         <f t="shared" si="7"/>
-        <v>https://www.velbert-autoverwertung.de</v>
+        <v>https://www.wuppertal-autoverwertung.de</v>
       </c>
       <c r="B362" t="s">
         <v>361</v>
-      </c>
-    </row>
-    <row r="363" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A363" t="str">
-        <f t="shared" si="7"/>
-        <v>https://www.wuppertal-autoverwertung.de</v>
-      </c>
-      <c r="B363" t="s">
-        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>